<commit_message>
docs: modelo de negocio completo - canvas maquetado, respuestas de actividad 1 y presentacion nueva
</commit_message>
<xml_diff>
--- a/docs/actividad-1/canvas-modelo-negocio.xlsx
+++ b/docs/actividad-1/canvas-modelo-negocio.xlsx
@@ -26,24 +26,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Georgia"/>
-      <b val="1"/>
-      <color rgb="001B2A4A"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="Georgia"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001E1B18"/>
-      <sz val="10"/>
+      <color rgb="0017293D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="000F2540"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -52,20 +52,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F0E8"/>
-        <bgColor rgb="00F5F0E8"/>
+        <fgColor rgb="000F2540"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="008B2635"/>
-        <bgColor rgb="008B2635"/>
+        <fgColor rgb="00F4F7FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B8960C"/>
-        <bgColor rgb="00B8960C"/>
+        <fgColor rgb="00E8F1FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF6E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F7EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDECEC"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,35 +91,42 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="001B2A4A"/>
+        <color rgb="009BB0C9"/>
       </left>
       <right style="thin">
-        <color rgb="001B2A4A"/>
+        <color rgb="009BB0C9"/>
       </right>
       <top style="thin">
-        <color rgb="001B2A4A"/>
+        <color rgb="009BB0C9"/>
       </top>
       <bottom style="thin">
-        <color rgb="001B2A4A"/>
+        <color rgb="009BB0C9"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -474,196 +493,470 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="46" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Business Model Canvas — Enlyce CRM Inmobiliario</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
+          <t>BUSINESS MODEL CANVAS  |  ENLYCE - CRM Inmobiliario para micro-inmobiliarias colombianas
+Cliente ancla: L&amp;C Propiedad Raíz (Medellín)  -  Agosto 2026  -  Ingeniería de Software</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Socios Clave</t>
-        </is>
-      </c>
+          <t>1. SOCIOS CLAVE
+- L&amp;C Propiedad Raíz: cliente ancla, valida requisitos y aporta datos reales.
+- Microsoft Azure / .NET: hosting e infraestructura del stack.
+- Meta - WhatsApp Business API: canal principal de captación de leads.
+- Proveedor de correo transaccional (SendGrid): alertas y notificaciones.
+- Universidad: soporte académico, asesoría y validación del proyecto.
+- Comunidad open source: PostgreSQL, EF Core, React/Vite.
+- SIC (marco regulatorio): registro RNBD y política de tratamiento.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Actividades Clave</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Propuesta de Valor</t>
-        </is>
-      </c>
+          <t>2. ACTIVIDADES CLAVE
+- Desarrollo del CRM (Clean Architecture, 172 tests automatizados).
+- Onboarding e implantación en menos de 24 horas.
+- Configuración del pipeline y de las etapas por inmobiliaria.
+- Capacitación de asesores (2 h) y soporte en español.
+- Mantener el cumplimiento de la Ley 1581 (consentimiento, política, auditoría).
+- Evolución del producto con feedback del cliente ancla.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>3. PROPUESTA DE VALOR
+"El CRM con el que una micro-inmobiliaria colombiana deja de perder leads."
+- Multi-asesor desde el dia 1: cada lead tiene dueño, nadie se pisa el cliente.
+- Pipeline Kanban visible: Contacto &gt; Visita &gt; Propuesta &gt; Negociación &gt; Cierre.
+- Alertas de seguimiento: el lead sin gestión se vuelve visible, no se pierde.
+- Cumplimiento de la Ley 1581 integrado, no como un anexo: consentimiento obligatorio,
+  política versionada, registro de auditoría y derechos del titular.
+- Baja lógica con auditoría: nada se borra, todo queda trazado.
+- Precio intermedio (~$158.000/mes) entre el gratuito sin valor y el costoso inaccesible.
+- Operativo en menos de 24 horas, 100 % en español colombiano.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Relacion con Clientes</t>
-        </is>
-      </c>
+          <t>4. RELACIÓN CON CLIENTES
+- Acompanamiento personal en la implantación (setup + capacitación).
+- Soporte directo por WhatsApp y correo, en horario laboral colombiano.
+- Co-creación con el cliente ancla: sus necesidades marcan el roadmap.
+- Autoservicio en la aplicación: el asesor gestiona su propio pipeline.
+- Actualizaciones continuas sin costo ni interrupción del servicio.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Segmentos de Clientes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="220" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>- Microsoft (Azure, .NET)
-- Meta (WhatsApp Business API)
-- PostgreSQL (open source)
-- L&amp;C Propiedad Raiz (cliente ancla)
-- Universidad (proyecto academico)
-- SendGrid (email transaccional)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>- Desarrollo y mantenimiento del software
-- Onboarding de clientes (&lt; 24h)
-- Soporte tecnico en espanol
-- Configuracion de pipelines
-- Cumplimiento normativo (Ley 1581)
-- Capacitacion de asesores</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>- CRM multi-agente para micro-inmobiliarias
-- Pipeline Kanban visual
-- Setup en menos de 1 dia
-- Cumplimiento Ley 1581 integrado
-- Interfaz 100% espanol colombiano
-- Precio accesible (~$158k/mes equipo)
-- Asignacion automatica de leads</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>- Onboarding personalizado (2h setup)
-- Soporte via WhatsApp/email
-- Capacitacion continua
-- Feedback loop con cliente ancla
-- Actualizaciones automaticas
-- Documentacion en espanol</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>- Micro-inmobiliarias (1-8 asesores)
-- Inmobiliarias &lt; 50 inmuebles
-- Medellin / area metropolitana
-- Clientes con Wasi gratis actual
-- Asesores independientes
-- Franchises pequenas</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="100" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Fuentes de Ingreso</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>1. Suscripcion mensual por equipo: $89.000 (base, 3 asesores)
-2. Asesor adicional: $19.000/mes
-3. Setup inicial: $150.000 (unico)
-4. Add-on WhatsApp API: $45.000/mes
-5. Add-on Portal web: $35.000/mes
-6. Add-on Reportes avanzados: $25.000/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="100" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Estructura de Costos</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>1. Hosting Azure/App Service: $120k-$200k/mes
-2. Dominio .com: ~$4k/mes
-3. WhatsApp API: variable por conversacion
-4. Email transaccional (SendGrid): $0-$15k/mes
-5. Monitoreo (Sentry): $0-$20k/mes
-6. Desarrollo: 96h (sunk cost, estudiante)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="100" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Recursos Clave</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>- Stack tecnico: ASP.NET Core 10, EF Core, PostgreSQL, React/Vite
-- Arquitectura Clean/Hexagonal (ardalis)
-- Conocimiento del mercado inmobiliario colombiano
-- Base de datos de leads e inmuebles de LYC
-- Infraestructura cloud (Azure)
-- Herramientas: GitHub, Visual Studio Community</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="100" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Canales</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>- Web app (React/Vite, responsive)
-- WhatsApp Business (comunicacion)
-- Email transaccional (onboarding, alertas)
-- Demo personalizada (reunion remota)
-- Referidos de cliente ancla (LYC)
-- Presencia universitaria (proyecto)</t>
-        </is>
-      </c>
-    </row>
+          <t>5. SEGMENTOS DE CLIENTES
+SEGMENTO PRINCIPAL
+- Inmobiliarias independientes de Medellín y su área metropolitana.
+- De 1 a 8 asesores comerciales, menos de 50 inmuebles activos.
+- Hoy operan con Wasi gratis, Excel y WhatsApp sin orden.
+- Facturación anual entre $100 M y $2.000 M COP.
+SEGMENTOS SECUNDARIOS
+- Asesores independientes que van a formar equipo.
+- Franquicias locales de inmobiliarias grandes que necesitan autonomia.
+- Constructoras pequeñas con venta directa.
+NO ES CLIENTE
+- Inmobiliarias de más de 15 asesores (les sirve Tokko).</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="3" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="3" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>6. RECURSOS CLAVE
+- Plataforma propia: ASP.NET Core 10 + EF Core + PostgreSQL + React/Vite.
+- Arquitectura hexagonal/limpia: dominio sin dependencias, portable y testeable.
+- Módulo de cumplimiento Ley 1581 (consentimientos, política versionada, auditoría).
+- Base de leads, inmuebles y propietarios de LYC.
+- Conocimiento del mercado inmobiliario de Medellín.
+- Equipo de desarrollo y su tiempo (96 h/semestre).</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>7. CANALES
+- Aplicación web responsive (React/Vite) - canal principal de uso.
+- WhatsApp Business - captación de leads y soporte.
+- Correo transaccional - alertas, seguimientos y onboarding.
+- Demostración personalizada (reunión presencial o remota).
+- Referidos del cliente ancla y del gremio inmobiliario local.
+- Vitrina académica del proyecto universitario.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="3" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="3" t="n"/>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>9. ESTRUCTURA DE COSTOS
+- Hosting Azure App Service + PostgreSQL administrado: $120.000 - $200.000 / mes.
+- Dominio y certificados: ~$4.000 / mes (SSL gratuito con Let's Encrypt).
+- WhatsApp Business API: variable, por conversación (Meta).
+- Correo transaccional y monitoreo: $0 - $35.000 / mes (planes gratuitos iniciales).
+- Desarrollo y mantenimiento: 96 h/semestre (costo hundido - proyecto académico).
+- Soporte y capacitación: horas de asesor por cliente nuevo.
+Costo fijo mensual estimado: $125.000 - $240.000. Es un modelo dirigido por el valor
+(no por el costo): margen positivo desde el segundo cliente.</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>8. FUENTES DE INGRESO
+1. Suscripción base por equipo (hasta 3 asesores): $89.000 / mes.
+2. Asesor adicional: $19.000 / mes cada uno (máximo 8).
+3. Implantación inicial (migración + capacitación): $150.000, pago único.
+4. Complemento WhatsApp Business API: $45.000 / mes.
+5. Complemento portal web público de inmuebles: $35.000 / mes.
+6. Complemento de reportes avanzados (PDF/Excel): $25.000 / mes.
+Caso tipico LYC (4 asesores): $158.000 / mes recurrentes + $150.000 de implantación.
+Meta del semestre: 10 clientes -&gt; MRR de $1.580.000 COP.</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="3" t="n"/>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="3" t="n"/>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="n"/>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="3" t="n"/>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="3" t="n"/>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="3" t="n"/>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="3" t="n"/>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="n"/>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="3" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="3" t="n"/>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="3" t="n"/>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+    </row>
+    <row r="28" ht="15" customHeight="1"/>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Restricción transversal: la Ley 1581 de 2012 exige autorización previa, expresa e informada del titular. En Enlyce ningún lead se crea sin consentimiento registrado, y toda operación queda en el log de auditoría.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31" ht="15" customHeight="1"/>
+    <row r="32" ht="15" customHeight="1"/>
+    <row r="33" ht="15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="F6:I6"/>
+  <mergeCells count="11">
+    <mergeCell ref="A2:B17"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="C2:D9"/>
+    <mergeCell ref="E2:F17"/>
+    <mergeCell ref="I2:J17"/>
+    <mergeCell ref="C10:D17"/>
+    <mergeCell ref="F18:J27"/>
+    <mergeCell ref="G10:H17"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A18:E27"/>
+    <mergeCell ref="G2:H9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>